<commit_message>
Resolve Russian tarot mapping conflicts
</commit_message>
<xml_diff>
--- a/outputs/019f2e9a-7504-7ee0-9b75-0d4456667415/russian_tarot_deck_tracker.xlsx
+++ b/outputs/019f2e9a-7504-7ee0-9b75-0d4456667415/russian_tarot_deck_tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Russian tarot" sheetId="1" r:id="R3f19722ed8cb4c17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Russian tarot" sheetId="1" r:id="R83f43eb14fc840ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,7 +131,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RussianTarotMappings" displayName="RussianTarotMappings" ref="A7:I97" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RussianTarotMappings" displayName="RussianTarotMappings" ref="A7:I92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Tarot card"/>
     <x:tableColumn id="2" name="Mapped card"/>
@@ -368,16 +368,16 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>59 uniquely mapped</x:v>
+        <x:v>64 uniquely mapped</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>12 conflicts</x:v>
+        <x:v>7 conflicts</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
         <x:v>7 open</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>2 missing art</x:v>
+        <x:v>0 missing art</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
@@ -591,238 +591,227 @@
         <x:v>The Chariot</x:v>
       </x:c>
       <x:c r="B15" s="7" t="str">
-        <x:v>VERA-7</x:v>
+        <x:v>Buran Breaks The Boundary</x:v>
       </x:c>
       <x:c r="C15" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D15" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-the-chariot-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-buran-breaks-the-boundary-the-chariot-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F15" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G15" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H15" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I15" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I15" s="8" t="str">
+        <x:v>Event art expresses The Chariot through Vera riding Buran at speed through opposing aurora and snow forces, with the village behind them, the breach ahead, and no literal wheeled chariot.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="7" t="str">
-        <x:v>The Chariot</x:v>
+        <x:v>Strength</x:v>
       </x:c>
       <x:c r="B16" s="7" t="str">
-        <x:v>Buran Breaks The Boundary</x:v>
+        <x:v>Major Yuri Volkov</x:v>
       </x:c>
       <x:c r="C16" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-buran-breaks-the-boundary-the-chariot-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/major-yuri-volkov-strength-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F16" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G16" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H16" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I16" s="8" t="str">
-        <x:v>Event art expresses The Chariot through Vera riding Buran at speed through opposing aurora and snow forces, with the village behind them, the breach ahead, and no literal wheeled chariot.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I16" s="8" t="str"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="7" t="str">
-        <x:v>Strength</x:v>
+        <x:v>The Hermit</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>Major Yuri Volkov</x:v>
+        <x:v>Meteor Lantern</x:v>
       </x:c>
       <x:c r="C17" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D17" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/major-yuri-volkov-strength-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-meteor-lantern-the-hermit-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F17" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G17" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H17" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I17" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I17" s="8" t="str">
+        <x:v>Relic art centers one old handmade lantern with blackened iron, scratched glass, red thread, boundary charms, a black meteor-glass shard, and warm true light against aurora-lit snow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="7" t="str">
-        <x:v>Strength</x:v>
+        <x:v>Wheel Of Fortune</x:v>
       </x:c>
       <x:c r="B18" s="7" t="str">
-        <x:v>Bogatyr Walks Through Smoke</x:v>
+        <x:v>Seventeen Seconds</x:v>
       </x:c>
       <x:c r="C18" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D18" s="7" t="str">
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-bogatyr-walks-through-smoke-strength-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-seventeen-seconds-wheel-of-fortune-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F18" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G18" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I18" s="8" t="str"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="7" t="str">
-        <x:v>The Hermit</x:v>
-      </x:c>
-      <x:c r="B19" s="7" t="str">
-        <x:v>Meteor Lantern</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D19" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-meteor-lantern-the-hermit-relic-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F19" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
+        <x:v>Justice</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="str"/>
+      <x:c r="C19" s="7" t="str"/>
+      <x:c r="D19" s="7" t="str"/>
+      <x:c r="E19" s="9" t="str"/>
+      <x:c r="F19" s="7" t="str"/>
       <x:c r="G19" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H19" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I19" s="8" t="str">
-        <x:v>Relic art centers one old handmade lantern with blackened iron, scratched glass, red thread, boundary charms, a black meteor-glass shard, and warm true light against aurora-lit snow.</x:v>
-      </x:c>
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="str"/>
+      <x:c r="I19" s="8" t="str"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="7" t="str">
-        <x:v>Wheel Of Fortune</x:v>
+        <x:v>The Hanged Man</x:v>
       </x:c>
       <x:c r="B20" s="7" t="str">
-        <x:v>Seventeen Seconds</x:v>
+        <x:v>Pavel Sokolov</x:v>
       </x:c>
       <x:c r="C20" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D20" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-seventeen-seconds-wheel-of-fortune-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/pavel-sokolov-the-hanged-man-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F20" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G20" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H20" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I20" s="8" t="str"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="7" t="str">
-        <x:v>Wheel Of Fortune</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="str">
-        <x:v>Radio Snow Speaks</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="str">
-        <x:v>Winter Front</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-radio-snow-speaks-wheel-of-fortune-event-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
+        <x:v>Death</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="str"/>
+      <x:c r="C21" s="7" t="str"/>
+      <x:c r="D21" s="7" t="str"/>
+      <x:c r="E21" s="9" t="str"/>
+      <x:c r="F21" s="7" t="str"/>
       <x:c r="G21" s="7" t="str">
-        <x:v>Conflict</x:v>
-      </x:c>
-      <x:c r="H21" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H21" s="7" t="str"/>
       <x:c r="I21" s="8" t="str"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="7" t="str">
-        <x:v>Justice</x:v>
-      </x:c>
-      <x:c r="B22" s="7" t="str"/>
-      <x:c r="C22" s="7" t="str"/>
-      <x:c r="D22" s="7" t="str"/>
-      <x:c r="E22" s="9" t="str"/>
-      <x:c r="F22" s="7" t="str"/>
+        <x:v>Temperance</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>Anya Lebedeva / Signal Escape Artist</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Closed City</x:v>
+      </x:c>
+      <x:c r="D22" s="7" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="E22" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-lebedeva-signal-escape-artist-temperance-character-card-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
+      <x:c r="F22" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G22" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H22" s="7" t="str"/>
-      <x:c r="I22" s="8" t="str"/>
+        <x:v>Conflict</x:v>
+      </x:c>
+      <x:c r="H22" s="7" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I22" s="8" t="str">
+        <x:v>Temperance was checked open in the Russian tarot tracker before assignment. Art should show Anya balancing two signals, two vessels, or two realities inside a sealed Closed City threshold, with analog relay cabinets, warning lamps, condensation, and an impossible corridor opening toward aurora-lit snow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="7" t="str">
-        <x:v>The Hanged Man</x:v>
+        <x:v>Temperance</x:v>
       </x:c>
       <x:c r="B23" s="7" t="str">
-        <x:v>Pavel Sokolov</x:v>
+        <x:v>Marya Zima</x:v>
       </x:c>
       <x:c r="C23" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D23" s="7" t="str">
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/pavel-sokolov-the-hanged-man-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/marya-zima-field-nurse-temperance-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F23" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G23" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H23" s="7" t="str">
         <x:v>Draft</x:v>
@@ -831,34 +820,47 @@
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="7" t="str">
-        <x:v>Death</x:v>
-      </x:c>
-      <x:c r="B24" s="7" t="str"/>
-      <x:c r="C24" s="7" t="str"/>
-      <x:c r="D24" s="7" t="str"/>
-      <x:c r="E24" s="9" t="str"/>
-      <x:c r="F24" s="7" t="str"/>
+        <x:v>The Devil</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="str">
+        <x:v>Karpova's Black Key</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="str">
+        <x:v>Closed City</x:v>
+      </x:c>
+      <x:c r="D24" s="7" t="str">
+        <x:v>Relic</x:v>
+      </x:c>
+      <x:c r="E24" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-karpovas-black-key-the-devil-relic-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G24" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H24" s="7" t="str"/>
+        <x:v>Conflict</x:v>
+      </x:c>
+      <x:c r="H24" s="7" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
       <x:c r="I24" s="8" t="str"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="7" t="str">
-        <x:v>Temperance</x:v>
+        <x:v>The Devil</x:v>
       </x:c>
       <x:c r="B25" s="7" t="str">
-        <x:v>Anya Lebedeva / Signal Escape Artist</x:v>
+        <x:v>Enemy Cache Unearthed</x:v>
       </x:c>
       <x:c r="C25" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D25" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-lebedeva-signal-escape-artist-temperance-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-enemy-cache-unearthed-the-devil-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F25" s="7" t="str">
@@ -870,60 +872,58 @@
       <x:c r="H25" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I25" s="8" t="str">
-        <x:v>Temperance was checked open in the Russian tarot tracker before assignment. Art should show Anya balancing two signals, two vessels, or two realities inside a sealed Closed City threshold, with analog relay cabinets, warning lamps, condensation, and an impossible corridor opening toward aurora-lit snow.</x:v>
-      </x:c>
+      <x:c r="I25" s="8" t="str"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="7" t="str">
-        <x:v>Temperance</x:v>
+        <x:v>The Tower</x:v>
       </x:c>
       <x:c r="B26" s="7" t="str">
-        <x:v>Marya Zima</x:v>
+        <x:v>Closed City Incident</x:v>
       </x:c>
       <x:c r="C26" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D26" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/marya-zima-field-nurse-temperance-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-incident-the-tower-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F26" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G26" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I26" s="8" t="str"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="7" t="str">
-        <x:v>The Devil</x:v>
+        <x:v>The Star</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>Karpova's Black Key</x:v>
+        <x:v>Nadia Belaya</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D27" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-karpovas-black-key-the-devil-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/nadia-belaya-the-star-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F27" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G27" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H27" s="7" t="str">
         <x:v>Approved</x:v>
@@ -932,19 +932,19 @@
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="7" t="str">
-        <x:v>The Devil</x:v>
+        <x:v>The Moon</x:v>
       </x:c>
       <x:c r="B28" s="7" t="str">
-        <x:v>Enemy Cache Unearthed</x:v>
+        <x:v>Subject 3: Zoya / Zoya Miranova</x:v>
       </x:c>
       <x:c r="C28" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D28" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-enemy-cache-unearthed-the-devil-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/subject-3-zoya-the-moon-character-card-art-corrected.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F28" s="7" t="str">
@@ -954,53 +954,55 @@
         <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I28" s="8" t="str"/>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I28" s="8" t="str">
+        <x:v>Corrected variant keeps the Closed City lab functional and humid rather than literally flooded; Moon symbolism comes from fogged glass, CRT crescents, lunar light, reflections, and hidden observer silhouettes.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="7" t="str">
-        <x:v>The Tower</x:v>
+        <x:v>The Moon</x:v>
       </x:c>
       <x:c r="B29" s="7" t="str">
-        <x:v>Closed City Incident</x:v>
+        <x:v>The Cabin Rite</x:v>
       </x:c>
       <x:c r="C29" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D29" s="7" t="str">
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-incident-the-tower-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-the-cabin-rite-the-moon-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F29" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G29" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H29" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I29" s="8" t="str"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="7" t="str">
-        <x:v>The Star</x:v>
+        <x:v>The Sun</x:v>
       </x:c>
       <x:c r="B30" s="7" t="str">
-        <x:v>Nadia Belaya</x:v>
+        <x:v>Reactor Prayer</x:v>
       </x:c>
       <x:c r="C30" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/nadia-belaya-the-star-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-reactor-prayer-the-sun-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F30" s="7" t="str">
@@ -1016,49 +1018,49 @@
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="7" t="str">
-        <x:v>The Moon</x:v>
+        <x:v>Judgement</x:v>
       </x:c>
       <x:c r="B31" s="7" t="str">
-        <x:v>Subject 3: Zoya / Zoya Miranova</x:v>
+        <x:v>The Meteor Wakes Under Snow</x:v>
       </x:c>
       <x:c r="C31" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D31" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/subject-3-zoya-the-moon-character-card-art-corrected.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-meteor-wakes-under-snow-judgement-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F31" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G31" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H31" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I31" s="8" t="str">
-        <x:v>Corrected variant keeps the Closed City lab functional and humid rather than literally flooded; Moon symbolism comes from fogged glass, CRT crescents, lunar light, reflections, and hidden observer silhouettes.</x:v>
+        <x:v>Event art centers the cracked meteor hollow, black glass fragments, tiny witnesses, and an aurora shaped like a natural calling horn with ghostly memory-figures rising through it.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="7" t="str">
-        <x:v>The Moon</x:v>
+        <x:v>The World</x:v>
       </x:c>
       <x:c r="B32" s="7" t="str">
-        <x:v>The Cabin Rite</x:v>
+        <x:v>The First Card Appears</x:v>
       </x:c>
       <x:c r="C32" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-the-cabin-rite-the-moon-event-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-the-world-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F32" s="7" t="str">
@@ -1068,32 +1070,32 @@
         <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H32" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I32" s="8" t="str"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="7" t="str">
-        <x:v>The Sun</x:v>
+        <x:v>The World</x:v>
       </x:c>
       <x:c r="B33" s="7" t="str">
-        <x:v>Reactor Prayer</x:v>
+        <x:v>Aal Luuk Mas Root</x:v>
       </x:c>
       <x:c r="C33" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D33" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-reactor-prayer-the-sun-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/aal-luuk-mas-root-the-world-rare-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F33" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G33" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H33" s="7" t="str">
         <x:v>Approved</x:v>
@@ -1102,10 +1104,10 @@
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="7" t="str">
-        <x:v>Judgement</x:v>
+        <x:v>Ace of Wands</x:v>
       </x:c>
       <x:c r="B34" s="7" t="str">
-        <x:v>The Meteor Wakes Under Snow</x:v>
+        <x:v>Aurora Opens Like A Door</x:v>
       </x:c>
       <x:c r="C34" s="7" t="str">
         <x:v>Far North</x:v>
@@ -1114,7 +1116,7 @@
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-meteor-wakes-under-snow-judgement-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-aurora-opens-like-a-door-ace-of-wands-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F34" s="7" t="str">
@@ -1127,114 +1129,119 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I34" s="8" t="str">
-        <x:v>Event art centers the cracked meteor hollow, black glass fragments, tiny witnesses, and an aurora shaped like a natural calling horn with ghostly memory-figures rising through it.</x:v>
+        <x:v>Event art uses one dominant vertical aurora column as a living wand/door, with snow, track lines, and black meteor glass reacting at the base while Buran remains a small answering presence.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="7" t="str">
-        <x:v>The World</x:v>
+        <x:v>Two of Wands</x:v>
       </x:c>
       <x:c r="B35" s="7" t="str">
-        <x:v>The First Card Appears</x:v>
+        <x:v>Volkov's Red Map</x:v>
       </x:c>
       <x:c r="C35" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D35" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-the-world-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-volkovs-red-map-two-of-wands-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F35" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G35" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H35" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I35" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I35" s="8" t="str">
+        <x:v>Approved relic art shows two black field rods over a red-stained command map, with Volkov's family/home traces and a face-down icon revealing the personal cost of choosing the impossible route.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>The World</x:v>
+        <x:v>Three of Wands</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
-        <x:v>Aal Luuk Mas Root</x:v>
+        <x:v>Radio Snow Speaks</x:v>
       </x:c>
       <x:c r="C36" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/aal-luuk-mas-root-the-world-rare-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-radio-snow-speaks-three-of-wands-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F36" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G36" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H36" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I36" s="8" t="str"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="7" t="str">
-        <x:v>Ace of Wands</x:v>
+        <x:v>Four of Wands</x:v>
       </x:c>
       <x:c r="B37" s="7" t="str">
-        <x:v>Aurora Opens Like A Door</x:v>
+        <x:v>Hearthstone Antler Crown</x:v>
       </x:c>
       <x:c r="C37" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D37" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E37" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-aurora-opens-like-a-door-ace-of-wands-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-hearthstone-antler-crown-four-of-wands-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F37" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G37" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H37" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I37" s="8" t="str">
-        <x:v>Event art uses one dominant vertical aurora column as a living wand/door, with snow, track lines, and black meteor glass reacting at the base while Buran remains a small answering presence.</x:v>
+        <x:v>Approved relic art shows the village celebration gathered around the ancient antler-and-stone relic, with four decorated posts forming the Four of Wands structure.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="7" t="str">
-        <x:v>Ace of Wands</x:v>
+        <x:v>Five of Wands</x:v>
       </x:c>
       <x:c r="B38" s="7" t="str">
-        <x:v>Black Snow Cartridge</x:v>
+        <x:v>Volkov Sends Another Wave</x:v>
       </x:c>
       <x:c r="C38" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D38" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E38" s="9" t="str"/>
+        <x:v>Event</x:v>
+      </x:c>
+      <x:c r="E38" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-volkov-sends-another-wave-five-of-wands-event-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
       <x:c r="F38" s="7" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Saved</x:v>
       </x:c>
       <x:c r="G38" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H38" s="7" t="str">
         <x:v>Draft</x:v>
@@ -1243,19 +1250,19 @@
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="7" t="str">
-        <x:v>Two of Wands</x:v>
+        <x:v>Six of Wands</x:v>
       </x:c>
       <x:c r="B39" s="7" t="str">
-        <x:v>Volkov's Red Map</x:v>
+        <x:v>Alexei Vranov / Cache-Born Hero</x:v>
       </x:c>
       <x:c r="C39" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D39" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E39" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-volkovs-red-map-two-of-wands-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/alexei-vranov-cache-born-hero-six-of-wands-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F39" s="7" t="str">
@@ -1268,15 +1275,15 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I39" s="8" t="str">
-        <x:v>Approved relic art shows two black field rods over a red-stained command map, with Volkov's family/home traces and a face-down icon revealing the personal cost of choosing the impossible route.</x:v>
+        <x:v>Rare Hero art shows Alexei with the black-and-gold Atlantean standard, Marya Zima as the female witness, and cross-area reflections tying pre-flood Atlantis, future Closed City, and the Far North meteor.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>Three of Wands</x:v>
+        <x:v>Seven of Wands</x:v>
       </x:c>
       <x:c r="B40" s="7" t="str">
-        <x:v>The Horizon Lens</x:v>
+        <x:v>The Ridge Rifle</x:v>
       </x:c>
       <x:c r="C40" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -1285,7 +1292,7 @@
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E40" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-horizon-lens-three-of-wands-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-ridge-rifle-seven-of-wands-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F40" s="7" t="str">
@@ -1298,24 +1305,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I40" s="8" t="str">
-        <x:v>Approved revision zooms into the cracked brass lens so the three visions appear only inside the glass, while the outside trench remains grounded and normal.</x:v>
+        <x:v>Approved relic art centers the sniper rifle as a defensive line object tied to Irina and the Winter Front ridge.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>Four of Wands</x:v>
+        <x:v>Eight of Wands</x:v>
       </x:c>
       <x:c r="B41" s="7" t="str">
-        <x:v>Hearthstone Antler Crown</x:v>
+        <x:v>Signal Array Turns</x:v>
       </x:c>
       <x:c r="C41" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D41" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E41" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-hearthstone-antler-crown-four-of-wands-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-signal-array-turns-eight-of-wands-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F41" s="7" t="str">
@@ -1327,25 +1334,23 @@
       <x:c r="H41" s="7" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="I41" s="8" t="str">
-        <x:v>Approved relic art shows the village celebration gathered around the ancient antler-and-stone relic, with four decorated posts forming the Four of Wands structure.</x:v>
-      </x:c>
+      <x:c r="I41" s="8" t="str"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="7" t="str">
-        <x:v>Five of Wands</x:v>
+        <x:v>Nine of Wands</x:v>
       </x:c>
       <x:c r="B42" s="7" t="str">
-        <x:v>Volkov Sends Another Wave</x:v>
+        <x:v>Oleg Baranov / Iron Strongman</x:v>
       </x:c>
       <x:c r="C42" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D42" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E42" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-volkov-sends-another-wave-five-of-wands-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/oleg-baranov-iron-strongman-nine-of-wands-character-card-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F42" s="7" t="str">
@@ -1357,14 +1362,16 @@
       <x:c r="H42" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I42" s="8" t="str"/>
+      <x:c r="I42" s="8" t="str">
+        <x:v>Corrected card art uses jet-black hair and beard for Oleg, and exactly nine vertical boundary stakes/poles to make the Nine of Wands mapping explicit.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="7" t="str">
-        <x:v>Six of Wands</x:v>
+        <x:v>Ten of Wands</x:v>
       </x:c>
       <x:c r="B43" s="7" t="str">
-        <x:v>Alexei Vranov / Cache-Born Hero</x:v>
+        <x:v>Rifle Company Soldier</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -1373,7 +1380,7 @@
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E43" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/alexei-vranov-cache-born-hero-six-of-wands-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/stepan-kuznetsov-rifle-company-soldier-ten-of-wands-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F43" s="7" t="str">
@@ -1385,25 +1392,23 @@
       <x:c r="H43" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I43" s="8" t="str">
-        <x:v>Rare Hero art shows Alexei with the black-and-gold Atlantean standard, Marya Zima as the female witness, and cross-area reflections tying pre-flood Atlantis, future Closed City, and the Far North meteor.</x:v>
-      </x:c>
+      <x:c r="I43" s="8" t="str"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="7" t="str">
-        <x:v>Seven of Wands</x:v>
+        <x:v>Page of Wands</x:v>
       </x:c>
       <x:c r="B44" s="7" t="str">
-        <x:v>The Ridge Rifle</x:v>
+        <x:v>Mila Vetrova / Gymnast</x:v>
       </x:c>
       <x:c r="C44" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D44" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E44" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-ridge-rifle-seven-of-wands-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/mila-vetrova-gymnast-page-of-wands-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F44" s="7" t="str">
@@ -1415,25 +1420,23 @@
       <x:c r="H44" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I44" s="8" t="str">
-        <x:v>Approved relic art centers the sniper rifle as a defensive line object tied to Irina and the Winter Front ridge.</x:v>
-      </x:c>
+      <x:c r="I44" s="8" t="str"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="7" t="str">
-        <x:v>Eight of Wands</x:v>
+        <x:v>Knight of Wands</x:v>
       </x:c>
       <x:c r="B45" s="7" t="str">
-        <x:v>Signal Array Turns</x:v>
+        <x:v>Buran / White Siberian Tiger</x:v>
       </x:c>
       <x:c r="C45" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D45" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E45" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-signal-array-turns-eight-of-wands-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/buran-white-siberian-tiger-knight-of-wands-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F45" s="7" t="str">
@@ -1443,16 +1446,16 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H45" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I45" s="8" t="str"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="7" t="str">
-        <x:v>Nine of Wands</x:v>
+        <x:v>Queen of Wands</x:v>
       </x:c>
       <x:c r="B46" s="7" t="str">
-        <x:v>Oleg Baranov / Iron Strongman</x:v>
+        <x:v>Vera Kargina / Meteor Spear</x:v>
       </x:c>
       <x:c r="C46" s="7" t="str">
         <x:v>Far North</x:v>
@@ -1461,7 +1464,7 @@
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E46" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/oleg-baranov-iron-strongman-nine-of-wands-character-card-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-kargina-meteor-spear-queen-of-wands-character-card-art-v3.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F46" s="7" t="str">
@@ -1474,15 +1477,15 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I46" s="8" t="str">
-        <x:v>Corrected card art uses jet-black hair and beard for Oleg, and exactly nine vertical boundary stakes/poles to make the Nine of Wands mapping explicit.</x:v>
+        <x:v>V3 keeps the younger, more vital Queen of Wands direction from v2 while adding red ribbons in Vera's hair and a practical riding harness on Buran to show their mount/leader relationship.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="7" t="str">
-        <x:v>Ten of Wands</x:v>
+        <x:v>King of Wands</x:v>
       </x:c>
       <x:c r="B47" s="7" t="str">
-        <x:v>Rifle Company Soldier</x:v>
+        <x:v>Bogatyr Champion</x:v>
       </x:c>
       <x:c r="C47" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -1491,7 +1494,7 @@
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E47" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/stepan-kuznetsov-rifle-company-soldier-ten-of-wands-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/ilya-voronin-bogatyr-champion-king-of-wands-character-card-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F47" s="7" t="str">
@@ -1507,19 +1510,19 @@
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="7" t="str">
-        <x:v>Page of Wands</x:v>
+        <x:v>Ace of Cups</x:v>
       </x:c>
       <x:c r="B48" s="7" t="str">
-        <x:v>Mila Vetrova / Gymnast</x:v>
+        <x:v>Hospital Orderly / Galina Reznik</x:v>
       </x:c>
       <x:c r="C48" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D48" s="7" t="str">
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E48" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/mila-vetrova-gymnast-page-of-wands-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/galina-reznik-hospital-orderly-ace-of-cups-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F48" s="7" t="str">
@@ -1531,23 +1534,25 @@
       <x:c r="H48" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I48" s="8" t="str"/>
+      <x:c r="I48" s="8" t="str">
+        <x:v>Ace of Cups was checked as unused in the Russian tarot tracker before assignment. The card should feel medical, intimate, and occult-scientific: a night ward, enamel basin, IV glass, iodine, black frost, and the suggestion that mercy itself is becoming a breach.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="7" t="str">
-        <x:v>Knight of Wands</x:v>
+        <x:v>Two of Cups</x:v>
       </x:c>
       <x:c r="B49" s="7" t="str">
-        <x:v>Buran / White Siberian Tiger</x:v>
+        <x:v>Tent Lights In The Whiteout</x:v>
       </x:c>
       <x:c r="C49" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D49" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E49" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/buran-white-siberian-tiger-knight-of-wands-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-tent-lights-in-the-whiteout-two-of-cups-event-art-v3.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F49" s="7" t="str">
@@ -1559,53 +1564,33 @@
       <x:c r="H49" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I49" s="8" t="str"/>
+      <x:c r="I49" s="8" t="str">
+        <x:v>V3 preserves Pavel and Mila sharing exactly two humble metal vodka cups in the tent light, keeps the established Sky-Hide Mirror looped frame, and makes the mirror feel more naturally grounded in the scene.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="7" t="str">
-        <x:v>Queen of Wands</x:v>
-      </x:c>
-      <x:c r="B50" s="7" t="str">
-        <x:v>Vera Kargina / Meteor Spear</x:v>
-      </x:c>
-      <x:c r="C50" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D50" s="7" t="str">
-        <x:v>Character</x:v>
-      </x:c>
-      <x:c r="E50" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-kargina-meteor-spear-queen-of-wands-character-card-art-v3.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F50" s="7" t="str">
-        <x:v>Saved</x:v>
+        <x:v>Three of Cups</x:v>
       </x:c>
       <x:c r="G50" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H50" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I50" s="8" t="str">
-        <x:v>V3 keeps the younger, more vital Queen of Wands direction from v2 while adding red ribbons in Vera's hair and a practical riding harness on Buran to show their mount/leader relationship.</x:v>
+        <x:v>Open</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="7" t="str">
-        <x:v>King of Wands</x:v>
+        <x:v>Four of Cups</x:v>
       </x:c>
       <x:c r="B51" s="7" t="str">
-        <x:v>Bogatyr Champion</x:v>
+        <x:v>The Village Refuses The Signal</x:v>
       </x:c>
       <x:c r="C51" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D51" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E51" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/ilya-voronin-bogatyr-champion-king-of-wands-character-card-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-village-refuses-the-signal-four-of-cups-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F51" s="7" t="str">
@@ -1617,23 +1602,25 @@
       <x:c r="H51" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I51" s="8" t="str"/>
+      <x:c r="I51" s="8" t="str">
+        <x:v>V2 shows collective village refusal through shutters closing, a radio being covered, charms turned inward, children guided away from windows, Pavel outside the social circle, and exactly four covered or overturned vessels in the foreground. The aurora is abstract rather than a literal cup.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="7" t="str">
-        <x:v>Ace of Cups</x:v>
+        <x:v>Five of Cups</x:v>
       </x:c>
       <x:c r="B52" s="7" t="str">
-        <x:v>Hospital Orderly / Galina Reznik</x:v>
+        <x:v>Marya's Thaw Cup</x:v>
       </x:c>
       <x:c r="C52" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D52" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E52" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/galina-reznik-hospital-orderly-ace-of-cups-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-maryas-thaw-cup-five-of-cups-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F52" s="7" t="str">
@@ -1646,15 +1633,15 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I52" s="8" t="str">
-        <x:v>Ace of Cups was checked as unused in the Russian tarot tracker before assignment. The card should feel medical, intimate, and occult-scientific: a night ward, enamel basin, IV glass, iodine, black frost, and the suggestion that mercy itself is becoming a breach.</x:v>
+        <x:v>Remapped from Temperance so Marya Zima keeps Temperance as a character. Approved relic art shows the glowing thaw cup in a frozen aid station with three fallen vessels and one standing background cup.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="7" t="str">
-        <x:v>Two of Cups</x:v>
+        <x:v>Six of Cups</x:v>
       </x:c>
       <x:c r="B53" s="7" t="str">
-        <x:v>Tent Lights In The Whiteout</x:v>
+        <x:v>Deep North Circus Arrives</x:v>
       </x:c>
       <x:c r="C53" s="7" t="str">
         <x:v>Far North</x:v>
@@ -1663,7 +1650,7 @@
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E53" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-tent-lights-in-the-whiteout-two-of-cups-event-art-v3.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-deep-north-circus-arrives-six-of-cups-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F53" s="7" t="str">
@@ -1676,15 +1663,15 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I53" s="8" t="str">
-        <x:v>V3 preserves Pavel and Mila sharing exactly two humble metal vodka cups in the tent light, keeps the established Sky-Hide Mirror looped frame, and makes the mirror feel more naturally grounded in the scene.</x:v>
+        <x:v>V2 corrects the visual count to exactly six cup-lanterns on one foreground crate and simplifies the circus-arrival tableau while keeping children drawn forward, elders uneasy, village houses, canvas tents, and aurora overhead.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="7" t="str">
-        <x:v>Three of Cups</x:v>
+        <x:v>Seven of Cups</x:v>
       </x:c>
       <x:c r="B54" s="7" t="str">
-        <x:v>The Sister-Vow Binding</x:v>
+        <x:v>Bogatyr's Relic Case</x:v>
       </x:c>
       <x:c r="C54" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -1693,7 +1680,7 @@
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E54" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-sister-vow-binding-three-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-bogatyrs-relic-case-seven-of-cups-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F54" s="7" t="str">
@@ -1705,25 +1692,23 @@
       <x:c r="H54" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I54" s="8" t="str">
-        <x:v>Approved relic art keeps exactly three cups in the warm memory scene, exactly three hanging cup-lockets, and Darya's long red-white prayer cloth wrapping through the charm and bayonet without showing a blunt end.</x:v>
-      </x:c>
+      <x:c r="I54" s="8" t="str"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="7" t="str">
-        <x:v>Four of Cups</x:v>
+        <x:v>Eight of Cups</x:v>
       </x:c>
       <x:c r="B55" s="7" t="str">
-        <x:v>The Village Refuses The Signal</x:v>
+        <x:v>The Rings Leave The Cabin</x:v>
       </x:c>
       <x:c r="C55" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D55" s="7" t="str">
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E55" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-village-refuses-the-signal-four-of-cups-event-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-the-rings-leave-the-cabin-eight-of-cups-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F55" s="7" t="str">
@@ -1735,25 +1720,23 @@
       <x:c r="H55" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I55" s="8" t="str">
-        <x:v>V2 shows collective village refusal through shutters closing, a radio being covered, charms turned inward, children guided away from windows, Pavel outside the social circle, and exactly four covered or overturned vessels in the foreground. The aurora is abstract rather than a literal cup.</x:v>
-      </x:c>
+      <x:c r="I55" s="8" t="str"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="7" t="str">
-        <x:v>Five of Cups</x:v>
+        <x:v>Nine of Cups</x:v>
       </x:c>
       <x:c r="B56" s="7" t="str">
-        <x:v>Marya's Thaw Cup</x:v>
+        <x:v>Karpova's Velvet Decanter</x:v>
       </x:c>
       <x:c r="C56" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D56" s="7" t="str">
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-maryas-thaw-cup-five-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-karpovas-velvet-decanter-nine-of-cups-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F56" s="7" t="str">
@@ -1763,57 +1746,35 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H56" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I56" s="8" t="str">
-        <x:v>Remapped from Temperance so Marya Zima keeps Temperance as a character. Approved relic art shows the glowing thaw cup in a frozen aid station with three fallen vessels and one standing background cup.</x:v>
+        <x:v>Approved relic art centers a crystal decanter in Karpova's private suite with exactly nine glasses/cup cues, burgundy velvet, occult-science papers, the Black Key, and cold reactor lights beyond the glass.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="7" t="str">
-        <x:v>Six of Cups</x:v>
-      </x:c>
-      <x:c r="B57" s="7" t="str">
-        <x:v>Deep North Circus Arrives</x:v>
-      </x:c>
-      <x:c r="C57" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D57" s="7" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="E57" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-deep-north-circus-arrives-six-of-cups-event-art-v2.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F57" s="7" t="str">
-        <x:v>Saved</x:v>
+        <x:v>Ten of Cups</x:v>
       </x:c>
       <x:c r="G57" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H57" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I57" s="8" t="str">
-        <x:v>V2 corrects the visual count to exactly six cup-lanterns on one foreground crate and simplifies the circus-arrival tableau while keeping children drawn forward, elders uneasy, village houses, canvas tents, and aurora overhead.</x:v>
+        <x:v>Open</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="7" t="str">
-        <x:v>Seven of Cups</x:v>
+        <x:v>Page of Cups</x:v>
       </x:c>
       <x:c r="B58" s="7" t="str">
-        <x:v>Bogatyr's Relic Case</x:v>
+        <x:v>Meteor Contact To The North</x:v>
       </x:c>
       <x:c r="C58" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D58" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E58" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-bogatyrs-relic-case-seven-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-meteor-contact-to-the-north-page-of-cups-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F58" s="7" t="str">
@@ -1829,19 +1790,19 @@
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="7" t="str">
-        <x:v>Eight of Cups</x:v>
+        <x:v>Knight of Cups</x:v>
       </x:c>
       <x:c r="B59" s="7" t="str">
-        <x:v>The Rings Leave The Cabin</x:v>
+        <x:v>Belorog / Aurora Reindeer</x:v>
       </x:c>
       <x:c r="C59" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D59" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E59" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-the-rings-leave-the-cabin-eight-of-cups-event-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/belorog-aurora-reindeer-knight-of-cups-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F59" s="7" t="str">
@@ -1853,23 +1814,25 @@
       <x:c r="H59" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I59" s="8" t="str"/>
+      <x:c r="I59" s="8" t="str">
+        <x:v>Knight of Cups was checked open in the Russian tarot tracker before assignment. Art should show a pale aurora-lit reindeer with luminous antlers, practical northern harness, red thread and charms, frozen river reflections, and a humble cup or bowl motif tied to spiritual passage.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="7" t="str">
-        <x:v>Nine of Cups</x:v>
+        <x:v>Queen of Cups</x:v>
       </x:c>
       <x:c r="B60" s="7" t="str">
-        <x:v>Karpova's Velvet Decanter</x:v>
+        <x:v>Aksinya Morozova / Frost Seer</x:v>
       </x:c>
       <x:c r="C60" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D60" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E60" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-karpovas-velvet-decanter-nine-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/aksinya-morozova-frost-seer-queen-of-cups-character-card-art-v4.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F60" s="7" t="str">
@@ -1879,18 +1842,18 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H60" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I60" s="8" t="str">
-        <x:v>Approved relic art centers a crystal decanter in Karpova's private suite with exactly nine glasses/cup cues, burgundy velvet, occult-science papers, the Black Key, and cold reactor lights beyond the glass.</x:v>
+        <x:v>V4 keeps the clear scrying reflection and hidden frost influence from v3 while improving continuity with Nadia Belaya's approved artwork: hooded off-white robe, red embroidery, brown braid, pendant, and warm Star-like healing light as she saves Pavel.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="7" t="str">
-        <x:v>Ten of Cups</x:v>
+        <x:v>King of Cups</x:v>
       </x:c>
       <x:c r="B61" s="7" t="str">
-        <x:v>The Hearth-Locket Pair</x:v>
+        <x:v>The Twin Waters Flask</x:v>
       </x:c>
       <x:c r="C61" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -1899,7 +1862,7 @@
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E61" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-hearth-locket-pair-ten-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-twin-waters-flask-king-of-cups-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F61" s="7" t="str">
@@ -1912,24 +1875,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I61" s="8" t="str">
-        <x:v>Approved relic art shows realistic paired lockets, Stepan's gloved hand holding Marya's portrait, Marya's nurse hand holding Stepan's portrait, and exactly ten cup motifs over a warm home vision.</x:v>
+        <x:v>Approved relic art shows a believable twin-chamber field flask with cold silver-blue dead water, warm golden living water, medical cloth, icon imagery, and restrained crown/cup authority.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="7" t="str">
-        <x:v>Page of Cups</x:v>
+        <x:v>Ace of Swords</x:v>
       </x:c>
       <x:c r="B62" s="7" t="str">
-        <x:v>Meteor Contact To The North</x:v>
+        <x:v>Meteor-Glass Spear</x:v>
       </x:c>
       <x:c r="C62" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D62" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E62" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-meteor-contact-to-the-north-page-of-cups-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-meteor-glass-spear-ace-of-swords-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F62" s="7" t="str">
@@ -1941,23 +1904,25 @@
       <x:c r="H62" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I62" s="8" t="str"/>
+      <x:c r="I62" s="8" t="str">
+        <x:v>Relic art focuses on a practical spear with a jagged black meteor-glass blade, red wraps, iron wire, protective knots, and aurora reflection at the village boundary.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="7" t="str">
-        <x:v>Knight of Cups</x:v>
+        <x:v>Two of Swords</x:v>
       </x:c>
       <x:c r="B63" s="7" t="str">
-        <x:v>Belorog / Aurora Reindeer</x:v>
+        <x:v>The Blind-Marked Kopeck</x:v>
       </x:c>
       <x:c r="C63" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D63" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E63" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/belorog-aurora-reindeer-knight-of-cups-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-blind-marked-kopeck-two-of-swords-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F63" s="7" t="str">
@@ -1967,27 +1932,27 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H63" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I63" s="8" t="str">
-        <x:v>Knight of Cups was checked open in the Russian tarot tracker before assignment. Art should show a pale aurora-lit reindeer with luminous antlers, practical northern harness, red thread and charms, frozen river reflections, and a humble cup or bowl motif tied to spiritual passage.</x:v>
+        <x:v>Approved art shows Irina, the suspended blind-marked coin, and exactly two crossed blades.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="7" t="str">
-        <x:v>Queen of Cups</x:v>
+        <x:v>Three of Swords</x:v>
       </x:c>
       <x:c r="B64" s="7" t="str">
-        <x:v>Aksinya Morozova / Frost Seer</x:v>
+        <x:v>Saint's Field Icon</x:v>
       </x:c>
       <x:c r="C64" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D64" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E64" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/aksinya-morozova-frost-seer-queen-of-cups-character-card-art-v4.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-saints-field-icon-three-of-swords-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F64" s="7" t="str">
@@ -2000,24 +1965,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I64" s="8" t="str">
-        <x:v>V4 keeps the clear scrying reflection and hidden frost influence from v3 while improving continuity with Nadia Belaya's approved artwork: hooded off-white robe, red embroidery, brown braid, pendant, and warm Star-like healing light as she saves Pavel.</x:v>
+        <x:v>Remapped from The Hierophant so Anastasia Lebedeva can keep formal faith authority. Approved relic art shows a cracked field icon crossed by three bayonet/sword wounds with rare white birds outside.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="7" t="str">
-        <x:v>King of Cups</x:v>
+        <x:v>Four of Swords</x:v>
       </x:c>
       <x:c r="B65" s="7" t="str">
-        <x:v>The Twin Waters Flask</x:v>
+        <x:v>Winter Stalls The War</x:v>
       </x:c>
       <x:c r="C65" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D65" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E65" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-twin-waters-flask-king-of-cups-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-winter-stalls-the-war-four-of-swords-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F65" s="7" t="str">
@@ -2029,25 +1994,23 @@
       <x:c r="H65" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I65" s="8" t="str">
-        <x:v>Approved relic art shows a believable twin-chamber field flask with cold silver-blue dead water, warm golden living water, medical cloth, icon imagery, and restrained crown/cup authority.</x:v>
-      </x:c>
+      <x:c r="I65" s="8" t="str"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="7" t="str">
-        <x:v>Ace of Swords</x:v>
+        <x:v>Five of Swords</x:v>
       </x:c>
       <x:c r="B66" s="7" t="str">
-        <x:v>Meteor-Glass Spear</x:v>
+        <x:v>The Knives Mark A False Road</x:v>
       </x:c>
       <x:c r="C66" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D66" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E66" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-meteor-glass-spear-ace-of-swords-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-knives-mark-a-false-road-five-of-swords-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F66" s="7" t="str">
@@ -2060,24 +2023,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I66" s="8" t="str">
-        <x:v>Relic art focuses on a practical spear with a jagged black meteor-glass blade, red wraps, iron wire, protective knots, and aurora reflection at the village boundary.</x:v>
+        <x:v>Event art centers Dmitri in the Deep North Circus tent with five dominant embedded blades on the target board, Pavel and Mila secondary in the snowy background, and the warning framed as both performance and deception.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="7" t="str">
-        <x:v>Two of Swords</x:v>
+        <x:v>Six of Swords</x:v>
       </x:c>
       <x:c r="B67" s="7" t="str">
-        <x:v>The Blind-Marked Kopeck</x:v>
+        <x:v>Frozen T-34</x:v>
       </x:c>
       <x:c r="C67" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D67" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E67" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-blind-marked-kopeck-two-of-swords-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/frozen-t34-six-of-swords-mount-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F67" s="7" t="str">
@@ -2087,27 +2050,27 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H67" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I67" s="8" t="str">
-        <x:v>Approved art shows Irina, the suspended blind-marked coin, and exactly two crossed blades.</x:v>
+        <x:v>Mount art uses the Frozen T-34 as a haunted ferry across the killing field, with wounded soldiers on the armor, exactly six sword-like bayonet markers lining the passage, and reactor-red convergence glow under the ice. It intentionally avoids Chariot charge language because Far North already uses that archetype.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="7" t="str">
-        <x:v>Three of Swords</x:v>
+        <x:v>Seven of Swords</x:v>
       </x:c>
       <x:c r="B68" s="7" t="str">
-        <x:v>Saint's Field Icon</x:v>
+        <x:v>Dmitri Voronov / Knife Thrower</x:v>
       </x:c>
       <x:c r="C68" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D68" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E68" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/winter-front-saints-field-icon-three-of-swords-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/dmitri-voronov-knife-thrower-seven-of-swords-character-card-art-v3.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F68" s="7" t="str">
@@ -2120,24 +2083,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I68" s="8" t="str">
-        <x:v>Remapped from The Hierophant so Anastasia Lebedeva can keep formal faith authority. Approved relic art shows a cracked field icon crossed by three bayonet/sword wounds with rare white birds outside.</x:v>
+        <x:v>V3 keeps Dmitri's longer dark hair and deep teal/emerald costume accents while improving the target-board knives with darker entry points, contact shadows, and visible wood damage so the blades read as embedded.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="7" t="str">
-        <x:v>Four of Swords</x:v>
+        <x:v>Eight of Swords</x:v>
       </x:c>
       <x:c r="B69" s="7" t="str">
-        <x:v>Winter Stalls The War</x:v>
+        <x:v>Subject 3 Wakes</x:v>
       </x:c>
       <x:c r="C69" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D69" s="7" t="str">
         <x:v>Event</x:v>
       </x:c>
       <x:c r="E69" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-winter-stalls-the-war-four-of-swords-event-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-subject-3-wakes-eight-of-swords-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F69" s="7" t="str">
@@ -2153,79 +2116,75 @@
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="7" t="str">
-        <x:v>Five of Swords</x:v>
+        <x:v>Nine of Swords</x:v>
       </x:c>
       <x:c r="B70" s="7" t="str">
-        <x:v>The Knives Mark A False Road</x:v>
+        <x:v>Cosmonaut Helmet With A Second Shadow</x:v>
       </x:c>
       <x:c r="C70" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D70" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E70" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-knives-mark-a-false-road-five-of-swords-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-swords-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F70" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G70" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H70" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I70" s="8" t="str">
-        <x:v>Event art centers Dmitri in the Deep North Circus tent with five dominant embedded blades on the target board, Pavel and Mila secondary in the snowy background, and the warning framed as both performance and deception.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I70" s="8" t="str"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="7" t="str">
-        <x:v>Six of Swords</x:v>
+        <x:v>Nine of Swords</x:v>
       </x:c>
       <x:c r="B71" s="7" t="str">
-        <x:v>Frozen T-34</x:v>
+        <x:v>Closed City Vision</x:v>
       </x:c>
       <x:c r="C71" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D71" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E71" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/frozen-t34-six-of-swords-mount-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-closed-city-vision-nine-of-swords-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F71" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G71" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H71" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I71" s="8" t="str">
-        <x:v>Mount art uses the Frozen T-34 as a haunted ferry across the killing field, with wounded soldiers on the armor, exactly six sword-like bayonet markers lining the passage, and reactor-red convergence glow under the ice. It intentionally avoids Chariot charge language because Far North already uses that archetype.</x:v>
-      </x:c>
+      <x:c r="I71" s="8" t="str"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="7" t="str">
-        <x:v>Seven of Swords</x:v>
+        <x:v>Ten of Swords</x:v>
       </x:c>
       <x:c r="B72" s="7" t="str">
-        <x:v>Dmitri Voronov / Knife Thrower</x:v>
+        <x:v>Bogatyr Walks Through Smoke</x:v>
       </x:c>
       <x:c r="C72" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D72" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E72" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/dmitri-voronov-knife-thrower-seven-of-swords-character-card-art-v3.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-bogatyr-walks-through-smoke-ten-of-swords-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F72" s="7" t="str">
@@ -2237,25 +2196,23 @@
       <x:c r="H72" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I72" s="8" t="str">
-        <x:v>V3 keeps Dmitri's longer dark hair and deep teal/emerald costume accents while improving the target-board knives with darker entry points, contact shadows, and visible wood damage so the blades read as embedded.</x:v>
-      </x:c>
+      <x:c r="I72" s="8" t="str"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="7" t="str">
-        <x:v>Eight of Swords</x:v>
+        <x:v>Page of Swords</x:v>
       </x:c>
       <x:c r="B73" s="7" t="str">
-        <x:v>Subject 3 Wakes</x:v>
+        <x:v>Redacted Incident Tape</x:v>
       </x:c>
       <x:c r="C73" s="7" t="str">
         <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D73" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E73" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-subject-3-wakes-eight-of-swords-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-redacted-incident-tape-page-of-swords-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F73" s="7" t="str">
@@ -2265,60 +2222,62 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H73" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I73" s="8" t="str"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="7" t="str">
-        <x:v>Nine of Swords</x:v>
+        <x:v>Knight of Swords</x:v>
       </x:c>
       <x:c r="B74" s="7" t="str">
-        <x:v>Cosmonaut Helmet With A Second Shadow</x:v>
+        <x:v>Darya Koval / Bayonet Saint</x:v>
       </x:c>
       <x:c r="C74" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D74" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E74" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-swords-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/darya-koval-bayonet-saint-knight-of-swords-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F74" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G74" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H74" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I74" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I74" s="8" t="str">
+        <x:v>Knight of Swords was checked open in the Russian tarot tracker before assignment. Art should show a fierce female Winter Front close-combat warrior with rifle and fixed bayonet, prayer cloth, diagonal snow/smoke motion, and occult trench lines breaking underfoot.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="7" t="str">
-        <x:v>Nine of Swords</x:v>
+        <x:v>Queen of Swords</x:v>
       </x:c>
       <x:c r="B75" s="7" t="str">
-        <x:v>Closed City Vision</x:v>
+        <x:v>Irina Sokolova</x:v>
       </x:c>
       <x:c r="C75" s="7" t="str">
         <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D75" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E75" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/winter-front-closed-city-vision-nine-of-swords-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/irina-sokolova-sniper-queen-of-swords-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F75" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G75" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H75" s="7" t="str">
         <x:v>Draft</x:v>
@@ -2327,25 +2286,40 @@
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="7" t="str">
-        <x:v>Ten of Swords</x:v>
-      </x:c>
-      <x:c r="B76" s="7" t="str"/>
-      <x:c r="C76" s="7" t="str"/>
-      <x:c r="D76" s="7" t="str"/>
-      <x:c r="E76" s="9" t="str"/>
-      <x:c r="F76" s="7" t="str"/>
+        <x:v>King of Swords</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="str">
+        <x:v>General Arkady Volkov / Army General</x:v>
+      </x:c>
+      <x:c r="C76" s="7" t="str">
+        <x:v>Winter Front</x:v>
+      </x:c>
+      <x:c r="D76" s="7" t="str">
+        <x:v>Character</x:v>
+      </x:c>
+      <x:c r="E76" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/arkady-volkov-army-general-king-of-swords-character-card-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
+      <x:c r="F76" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G76" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H76" s="7" t="str"/>
-      <x:c r="I76" s="8" t="str"/>
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="H76" s="7" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I76" s="8" t="str">
+        <x:v>Remapped from The Emperor so Colonel Viktor Semyonov can own the Emperor archetype. King of Swords centers Volkov's strategic cruelty, silver pointer-as-sword, red command sash, casualty lists, and soldiers sent into lethal snow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="7" t="str">
-        <x:v>Page of Swords</x:v>
+        <x:v>Ace of Pentacles</x:v>
       </x:c>
       <x:c r="B77" s="7" t="str">
-        <x:v>Redacted Incident Tape</x:v>
+        <x:v>Chintamani Fragment</x:v>
       </x:c>
       <x:c r="C77" s="7" t="str">
         <x:v>Closed City</x:v>
@@ -2354,118 +2328,125 @@
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E77" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-redacted-incident-tape-page-of-swords-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-chintamani-fragment-ace-of-pentacles-relic-art-corrected.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F77" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G77" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H77" s="7" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="I77" s="8" t="str"/>
+      <x:c r="I77" s="8" t="str">
+        <x:v>Corrected variant keeps the Chintamani fragment sealed inside the evidence container, with the tag and cord attached outside the latch/seal rather than passing through the glass.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="7" t="str">
-        <x:v>Page of Swords</x:v>
+        <x:v>Two of Pentacles</x:v>
       </x:c>
       <x:c r="B78" s="7" t="str">
-        <x:v>Frozen Field Radio</x:v>
+        <x:v>Circus Convergence Rings</x:v>
       </x:c>
       <x:c r="C78" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D78" s="7" t="str">
         <x:v>Relic</x:v>
       </x:c>
-      <x:c r="E78" s="9" t="str"/>
+      <x:c r="E78" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-circus-convergence-rings-two-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
       <x:c r="F78" s="7" t="str">
-        <x:v>Missing</x:v>
+        <x:v>Saved</x:v>
       </x:c>
       <x:c r="G78" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H78" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I78" s="8" t="str"/>
+      <x:c r="I78" s="8" t="str">
+        <x:v>Relic art shows exactly two dominant old iron circus rings with worn rope, red thread, leather wraps, subtle Atlantean etching, and Old Rite floor geometry inside the Deep North Circus tent.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="7" t="str">
-        <x:v>Knight of Swords</x:v>
+        <x:v>Three of Pentacles</x:v>
       </x:c>
       <x:c r="B79" s="7" t="str">
-        <x:v>Darya Koval / Bayonet Saint</x:v>
+        <x:v>Dream Monitors Synchronize</x:v>
       </x:c>
       <x:c r="C79" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D79" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E79" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/darya-koval-bayonet-saint-knight-of-swords-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-dream-monitors-synchronize-three-of-pentacles-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F79" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G79" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H79" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I79" s="8" t="str">
-        <x:v>Knight of Swords was checked open in the Russian tarot tracker before assignment. Art should show a fierce female Winter Front close-combat warrior with rifle and fixed bayonet, prayer cloth, diagonal snow/smoke motion, and occult trench lines breaking underfoot.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I79" s="8" t="str"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="7" t="str">
-        <x:v>Queen of Swords</x:v>
+        <x:v>Three of Pentacles</x:v>
       </x:c>
       <x:c r="B80" s="7" t="str">
-        <x:v>Irina Sokolova</x:v>
+        <x:v>The Circus Performs The Old Rite</x:v>
       </x:c>
       <x:c r="C80" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D80" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E80" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/irina-sokolova-sniper-queen-of-swords-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-pentacles-event-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F80" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G80" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H80" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I80" s="8" t="str"/>
+      <x:c r="I80" s="8" t="str">
+        <x:v>V2 shows Mila, Dmitri, and Oleg forming three centers of craft inside the tent, with a witnessing crowd and rope/lantern/floor geometry suggesting three interlocked rings around a vertical convergence mark. Dmitri and Oleg read as collaborators in the rite rather than opponents.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="7" t="str">
-        <x:v>King of Swords</x:v>
+        <x:v>Four of Pentacles</x:v>
       </x:c>
       <x:c r="B81" s="7" t="str">
-        <x:v>General Arkady Volkov / Army General</x:v>
+        <x:v>Lead-Sealed Notebook</x:v>
       </x:c>
       <x:c r="C81" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D81" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E81" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/arkady-volkov-army-general-king-of-swords-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F81" s="7" t="str">
@@ -2475,145 +2456,143 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H81" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I81" s="8" t="str">
-        <x:v>Remapped from The Emperor so Colonel Viktor Semyonov can own the Emperor archetype. King of Swords centers Volkov's strategic cruelty, silver pointer-as-sword, red command sash, casualty lists, and soldiers sent into lethal snow.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I81" s="8" t="str"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="7" t="str">
-        <x:v>Ace of Pentacles</x:v>
+        <x:v>Five of Pentacles</x:v>
       </x:c>
       <x:c r="B82" s="7" t="str">
-        <x:v>Chintamani Fragment</x:v>
+        <x:v>Semyonov Orders Silence</x:v>
       </x:c>
       <x:c r="C82" s="7" t="str">
         <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D82" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E82" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-chintamani-fragment-ace-of-pentacles-relic-art-corrected.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F82" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G82" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H82" s="7" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="I82" s="8" t="str">
-        <x:v>Corrected variant keeps the Chintamani fragment sealed inside the evidence container, with the tag and cord attached outside the latch/seal rather than passing through the glass.</x:v>
-      </x:c>
+      <x:c r="I82" s="8" t="str"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="7" t="str">
-        <x:v>Two of Pentacles</x:v>
+        <x:v>Five of Pentacles</x:v>
       </x:c>
       <x:c r="B83" s="7" t="str">
-        <x:v>Circus Convergence Rings</x:v>
+        <x:v>Nadia Finds The Survivor</x:v>
       </x:c>
       <x:c r="C83" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D83" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E83" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-circus-convergence-rings-two-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-five-of-pentacles-event-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F83" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G83" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Conflict</x:v>
       </x:c>
       <x:c r="H83" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I83" s="8" t="str">
-        <x:v>Relic art shows exactly two dominant old iron circus rings with worn rope, red thread, leather wraps, subtle Atlantean etching, and Old Rite floor geometry inside the Deep North Circus tent.</x:v>
+        <x:v>Event art keeps Nadia and Pavel continuity while distinguishing itself from Nadia's character card through wider composition, Pavel's exposure, the visible Sky-Hide Mirror, distant shelter lights, and the huge aurora wound overhead.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="7" t="str">
-        <x:v>Three of Pentacles</x:v>
+        <x:v>Six of Pentacles</x:v>
       </x:c>
       <x:c r="B84" s="7" t="str">
-        <x:v>Dream Monitors Synchronize</x:v>
+        <x:v>Civilian Evacuee / Anya Petrovna</x:v>
       </x:c>
       <x:c r="C84" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D84" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E84" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-dream-monitors-synchronize-three-of-pentacles-event-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F84" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G84" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H84" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I84" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I84" s="8" t="str">
+        <x:v>Card art shows Anya at a frozen evacuation road with a civilian sled, shared bread, a cracked icon with subtle reactor-red reflection, exactly six visible ration tokens, and a half-buried iron ring hinting at the later Deep North Circus connection. Six of Pentacles was checked open before assignment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="7" t="str">
-        <x:v>Three of Pentacles</x:v>
+        <x:v>Seven of Pentacles</x:v>
       </x:c>
       <x:c r="B85" s="7" t="str">
-        <x:v>The Circus Performs The Old Rite</x:v>
+        <x:v>Village Woodcutter / Tomas Yurin</x:v>
       </x:c>
       <x:c r="C85" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D85" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E85" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-pentacles-event-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F85" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G85" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H85" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I85" s="8" t="str">
-        <x:v>V2 shows Mila, Dmitri, and Oleg forming three centers of craft inside the tent, with a witnessing crowd and rope/lantern/floor geometry suggesting three interlocked rings around a vertical convergence mark. Dmitri and Oleg read as collaborators in the rite rather than opponents.</x:v>
+        <x:v>Seven of Pentacles was checked open in the Russian tarot tracker before assignment. Art should show a rugged village laborer with stacked firewood, sled runners, repaired boundary posts, and exactly seven visible cut log ends, carved post marks, or pentacle-like wood rounds as the tarot cue.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="7" t="str">
-        <x:v>Four of Pentacles</x:v>
+        <x:v>Eight of Pentacles</x:v>
       </x:c>
       <x:c r="B86" s="7" t="str">
-        <x:v>Lead-Sealed Notebook</x:v>
+        <x:v>Yakov Antonov / Winter Engineer</x:v>
       </x:c>
       <x:c r="C86" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D86" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E86" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F86" s="7" t="str">
@@ -2623,83 +2602,55 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H86" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
       </x:c>
       <x:c r="I86" s="8" t="str"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="7" t="str">
-        <x:v>Five of Pentacles</x:v>
-      </x:c>
-      <x:c r="B87" s="7" t="str">
-        <x:v>Semyonov Orders Silence</x:v>
-      </x:c>
-      <x:c r="C87" s="7" t="str">
-        <x:v>Closed City</x:v>
-      </x:c>
-      <x:c r="D87" s="7" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="E87" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F87" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
+        <x:v>Nine of Pentacles</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="str"/>
+      <x:c r="C87" s="7" t="str"/>
+      <x:c r="D87" s="7" t="str"/>
+      <x:c r="E87" s="9" t="str"/>
+      <x:c r="F87" s="7" t="str"/>
       <x:c r="G87" s="7" t="str">
-        <x:v>Conflict</x:v>
-      </x:c>
-      <x:c r="H87" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H87" s="7" t="str"/>
       <x:c r="I87" s="8" t="str"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="7" t="str">
-        <x:v>Five of Pentacles</x:v>
-      </x:c>
-      <x:c r="B88" s="7" t="str">
-        <x:v>Nadia Finds The Survivor</x:v>
-      </x:c>
-      <x:c r="C88" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D88" s="7" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="E88" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-five-of-pentacles-event-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F88" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
+        <x:v>Ten of Pentacles</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="str"/>
+      <x:c r="C88" s="7" t="str"/>
+      <x:c r="D88" s="7" t="str"/>
+      <x:c r="E88" s="9" t="str"/>
+      <x:c r="F88" s="7" t="str"/>
       <x:c r="G88" s="7" t="str">
-        <x:v>Conflict</x:v>
-      </x:c>
-      <x:c r="H88" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I88" s="8" t="str">
-        <x:v>Event art keeps Nadia and Pavel continuity while distinguishing itself from Nadia's character card through wider composition, Pavel's exposure, the visible Sky-Hide Mirror, distant shelter lights, and the huge aurora wound overhead.</x:v>
-      </x:c>
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="H88" s="7" t="str"/>
+      <x:c r="I88" s="8" t="str"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="7" t="str">
-        <x:v>Six of Pentacles</x:v>
+        <x:v>Page of Pentacles</x:v>
       </x:c>
       <x:c r="B89" s="7" t="str">
-        <x:v>Civilian Evacuee / Anya Petrovna</x:v>
+        <x:v>Sky-Hide Mirror</x:v>
       </x:c>
       <x:c r="C89" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D89" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E89" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F89" s="7" t="str">
@@ -2712,24 +2663,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I89" s="8" t="str">
-        <x:v>Card art shows Anya at a frozen evacuation road with a civilian sled, shared bread, a cracked icon with subtle reactor-red reflection, exactly six visible ration tokens, and a half-buried iron ring hinting at the later Deep North Circus connection. Six of Pentacles was checked open before assignment.</x:v>
+        <x:v>Remapped from Page of Cups to Page of Pentacles so Meteor Contact To The North can own the cup-message archetype. Corrected variant increases the mirror scale to match Pavel's character artwork, making it a large hand-held disc rather than a small pendant.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="7" t="str">
-        <x:v>Seven of Pentacles</x:v>
+        <x:v>Knight of Pentacles</x:v>
       </x:c>
       <x:c r="B90" s="7" t="str">
-        <x:v>Village Woodcutter / Tomas Yurin</x:v>
+        <x:v>Buran's Boundary Harness</x:v>
       </x:c>
       <x:c r="C90" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D90" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E90" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F90" s="7" t="str">
@@ -2742,24 +2693,24 @@
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I90" s="8" t="str">
-        <x:v>Seven of Pentacles was checked open in the Russian tarot tracker before assignment. Art should show a rugged village laborer with stacked firewood, sled runners, repaired boundary posts, and exactly seven visible cut log ends, carved post marks, or pentacle-like wood rounds as the tarot cue.</x:v>
+        <x:v>Relic art keeps the harness consistent with Buran and Vera's established imagery: rugged dark leather, iron rings, red cords, boundary charms, tiger pawprints, Vera's boot tracks, and aurora-lit village posts.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="7" t="str">
-        <x:v>Eight of Pentacles</x:v>
+        <x:v>Queen of Pentacles</x:v>
       </x:c>
       <x:c r="B91" s="7" t="str">
-        <x:v>Yakov Antonov / Winter Engineer</x:v>
+        <x:v>VERA-7</x:v>
       </x:c>
       <x:c r="C91" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D91" s="7" t="str">
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E91" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png","Open art")</x:f>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-queen-of-pentacles-character-card-art.png","Open art")</x:f>
         <x:v>Open art</x:v>
       </x:c>
       <x:c r="F91" s="7" t="str">
@@ -2769,156 +2720,51 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H91" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I91" s="8" t="str"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="7" t="str">
-        <x:v>Nine of Pentacles</x:v>
-      </x:c>
-      <x:c r="B92" s="7" t="str"/>
-      <x:c r="C92" s="7" t="str"/>
-      <x:c r="D92" s="7" t="str"/>
-      <x:c r="E92" s="9" t="str"/>
-      <x:c r="F92" s="7" t="str"/>
+        <x:v>King of Pentacles</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="str">
+        <x:v>Reactor Core Fragment</x:v>
+      </x:c>
+      <x:c r="C92" s="7" t="str">
+        <x:v>Closed City</x:v>
+      </x:c>
+      <x:c r="D92" s="7" t="str">
+        <x:v>Relic</x:v>
+      </x:c>
+      <x:c r="E92" s="9" t="str">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-reactor-core-fragment-king-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:v>Open art</x:v>
+      </x:c>
+      <x:c r="F92" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G92" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H92" s="7" t="str"/>
-      <x:c r="I92" s="8" t="str"/>
-    </x:row>
-    <x:row r="93" ht="23" customHeight="1">
-      <x:c r="A93" s="7" t="str">
-        <x:v>Ten of Pentacles</x:v>
-      </x:c>
-      <x:c r="B93" s="7" t="str"/>
-      <x:c r="C93" s="7" t="str"/>
-      <x:c r="D93" s="7" t="str"/>
-      <x:c r="E93" s="9" t="str"/>
-      <x:c r="F93" s="7" t="str"/>
-      <x:c r="G93" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H93" s="7" t="str"/>
-      <x:c r="I93" s="8" t="str"/>
-    </x:row>
-    <x:row r="94" ht="23" customHeight="1">
-      <x:c r="A94" s="7" t="str">
-        <x:v>Page of Pentacles</x:v>
-      </x:c>
-      <x:c r="B94" s="7" t="str">
-        <x:v>Sky-Hide Mirror</x:v>
-      </x:c>
-      <x:c r="C94" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D94" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E94" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F94" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G94" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H94" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I94" s="8" t="str">
-        <x:v>Remapped from Page of Cups to Page of Pentacles so Meteor Contact To The North can own the cup-message archetype. Corrected variant increases the mirror scale to match Pavel's character artwork, making it a large hand-held disc rather than a small pendant.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95" ht="23" customHeight="1">
-      <x:c r="A95" s="7" t="str">
-        <x:v>Knight of Pentacles</x:v>
-      </x:c>
-      <x:c r="B95" s="7" t="str">
-        <x:v>Buran's Boundary Harness</x:v>
-      </x:c>
-      <x:c r="C95" s="7" t="str">
-        <x:v>Far North</x:v>
-      </x:c>
-      <x:c r="D95" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E95" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F95" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G95" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H95" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I95" s="8" t="str">
-        <x:v>Relic art keeps the harness consistent with Buran and Vera's established imagery: rugged dark leather, iron rings, red cords, boundary charms, tiger pawprints, Vera's boot tracks, and aurora-lit village posts.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="23" customHeight="1">
-      <x:c r="A96" s="7" t="str">
-        <x:v>Queen of Pentacles</x:v>
-      </x:c>
-      <x:c r="B96" s="7" t="str"/>
-      <x:c r="C96" s="7" t="str"/>
-      <x:c r="D96" s="7" t="str"/>
-      <x:c r="E96" s="9" t="str"/>
-      <x:c r="F96" s="7" t="str"/>
-      <x:c r="G96" s="7" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H96" s="7" t="str"/>
-      <x:c r="I96" s="8" t="str"/>
-    </x:row>
-    <x:row r="97" ht="23" customHeight="1">
-      <x:c r="A97" s="7" t="str">
-        <x:v>King of Pentacles</x:v>
-      </x:c>
-      <x:c r="B97" s="7" t="str">
-        <x:v>Reactor Core Fragment</x:v>
-      </x:c>
-      <x:c r="C97" s="7" t="str">
-        <x:v>Closed City</x:v>
-      </x:c>
-      <x:c r="D97" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E97" s="9" t="str">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-reactor-core-fragment-king-of-pentacles-relic-art.png","Open art")</x:f>
-        <x:v>Open art</x:v>
-      </x:c>
-      <x:c r="F97" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G97" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H97" s="7" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="H92" s="7" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="I97" s="8" t="str">
+      <x:c r="I92" s="8" t="str">
         <x:v>Approved revision preserves the shard but replaces the paired gauges with a locked power pedestal, a single pentacle seal, and conduits carrying its energy into the Closed City.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="G8:G97">
+  <x:conditionalFormatting sqref="G8:G92">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Conflict"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Open"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F8:F97">
+  <x:conditionalFormatting sqref="F8:F92">
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Missing"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd365c26ae7e24329"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bf3c4d1e30743e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Russian tarot deck mapping
</commit_message>
<xml_diff>
--- a/outputs/019f2e9a-7504-7ee0-9b75-0d4456667415/russian_tarot_deck_tracker.xlsx
+++ b/outputs/019f2e9a-7504-7ee0-9b75-0d4456667415/russian_tarot_deck_tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Russian tarot" sheetId="1" r:id="R366b9de386bf441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Russian tarot" sheetId="1" r:id="R51e4040083eb4479"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,7 +131,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RussianTarotMappings" displayName="RussianTarotMappings" ref="A7:I87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RussianTarotMappings" displayName="RussianTarotMappings" ref="A7:I85" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Tarot card"/>
     <x:tableColumn id="2" name="Mapped card"/>
@@ -368,13 +368,13 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>74 uniquely mapped</x:v>
+        <x:v>78 uniquely mapped</x:v>
       </x:c>
       <x:c r="C5" s="3" t="str">
-        <x:v>2 conflicts</x:v>
+        <x:v>0 conflicts</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>2 open</x:v>
+        <x:v>0 open</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
         <x:v>0 missing art</x:v>
@@ -1505,8 +1505,30 @@
       <x:c r="A46" s="7" t="str">
         <x:v>Three of Cups</x:v>
       </x:c>
+      <x:c r="B46" s="7" t="str">
+        <x:v>The Circus Performs The Old Rite</x:v>
+      </x:c>
+      <x:c r="C46" s="7" t="str">
+        <x:v>Far North</x:v>
+      </x:c>
+      <x:c r="D46" s="7" t="str">
+        <x:v>Event</x:v>
+      </x:c>
+      <x:c r="E46" s="9" t="e">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-cups-event-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-cups-event-art.png, friendlyName=Open art</x:v>
+      </x:c>
+      <x:c r="F46" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G46" s="7" t="str">
-        <x:v>Open</x:v>
+        <x:v>Unique</x:v>
+      </x:c>
+      <x:c r="H46" s="7" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I46" s="8" t="str">
+        <x:v>Remapped from Three of Pentacles. Revised art uses exactly three ritual cups and a joined light pattern to express communal trust and celebration.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
@@ -1689,8 +1711,30 @@
       <x:c r="A53" s="7" t="str">
         <x:v>Ten of Cups</x:v>
       </x:c>
+      <x:c r="B53" s="7" t="str">
+        <x:v>Nadia Finds The Survivor</x:v>
+      </x:c>
+      <x:c r="C53" s="7" t="str">
+        <x:v>Far North</x:v>
+      </x:c>
+      <x:c r="D53" s="7" t="str">
+        <x:v>Event</x:v>
+      </x:c>
+      <x:c r="E53" s="9" t="e">
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-ten-of-cups-event-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-ten-of-cups-event-art.png, friendlyName=Open art</x:v>
+      </x:c>
+      <x:c r="F53" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
       <x:c r="G53" s="7" t="str">
-        <x:v>Open</x:v>
+        <x:v>Unique</x:v>
+      </x:c>
+      <x:c r="H53" s="7" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I53" s="8" t="str">
+        <x:v>Remapped from Five of Pentacles. Revised art uses exactly ten brighter stars, a gentle aurora, and a subdued mirror vision to foreshadow chosen family.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
@@ -2300,7 +2344,7 @@
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G74" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Unique</x:v>
       </x:c>
       <x:c r="H74" s="7" t="str">
         <x:v>Approved</x:v>
@@ -2309,56 +2353,54 @@
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="7" t="str">
-        <x:v>Three of Pentacles</x:v>
+        <x:v>Four of Pentacles</x:v>
       </x:c>
       <x:c r="B75" s="7" t="str">
-        <x:v>The Circus Performs The Old Rite</x:v>
+        <x:v>Lead-Sealed Notebook</x:v>
       </x:c>
       <x:c r="C75" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D75" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E75" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-pentacles-event-art-v2.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-the-circus-performs-the-old-rite-three-of-pentacles-event-art-v2.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F75" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G75" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H75" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I75" s="8" t="str">
-        <x:v>V2 shows Mila, Dmitri, and Oleg forming three centers of craft inside the tent, with a witnessing crowd and rope/lantern/floor geometry suggesting three interlocked rings around a vertical convergence mark. Dmitri and Oleg read as collaborators in the rite rather than opponents.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I75" s="8" t="str"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="7" t="str">
-        <x:v>Four of Pentacles</x:v>
+        <x:v>Five of Pentacles</x:v>
       </x:c>
       <x:c r="B76" s="7" t="str">
-        <x:v>Lead-Sealed Notebook</x:v>
+        <x:v>Semyonov Orders Silence</x:v>
       </x:c>
       <x:c r="C76" s="7" t="str">
         <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D76" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E76" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-lead-sealed-notebook-four-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F76" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G76" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Unique</x:v>
       </x:c>
       <x:c r="H76" s="7" t="str">
         <x:v>Approved</x:v>
@@ -2367,68 +2409,70 @@
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="7" t="str">
-        <x:v>Five of Pentacles</x:v>
+        <x:v>Six of Pentacles</x:v>
       </x:c>
       <x:c r="B77" s="7" t="str">
-        <x:v>Semyonov Orders Silence</x:v>
+        <x:v>Civilian Evacuee / Anya Petrovna</x:v>
       </x:c>
       <x:c r="C77" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Winter Front</x:v>
       </x:c>
       <x:c r="D77" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E77" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-semyonov-orders-silence-five-of-pentacles-event-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F77" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G77" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H77" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I77" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I77" s="8" t="str">
+        <x:v>Card art shows Anya at a frozen evacuation road with a civilian sled, shared bread, a cracked icon with subtle reactor-red reflection, exactly six visible ration tokens, and a half-buried iron ring hinting at the later Deep North Circus connection. Six of Pentacles was checked open before assignment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="7" t="str">
-        <x:v>Five of Pentacles</x:v>
+        <x:v>Seven of Pentacles</x:v>
       </x:c>
       <x:c r="B78" s="7" t="str">
-        <x:v>Nadia Finds The Survivor</x:v>
+        <x:v>Village Woodcutter / Tomas Yurin</x:v>
       </x:c>
       <x:c r="C78" s="7" t="str">
         <x:v>Far North</x:v>
       </x:c>
       <x:c r="D78" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E78" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-five-of-pentacles-event-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/far-north-nadia-finds-the-survivor-five-of-pentacles-event-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F78" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G78" s="7" t="str">
-        <x:v>Conflict</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H78" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="I78" s="8" t="str">
-        <x:v>Event art keeps Nadia and Pavel continuity while distinguishing itself from Nadia's character card through wider composition, Pavel's exposure, the visible Sky-Hide Mirror, distant shelter lights, and the huge aurora wound overhead.</x:v>
+        <x:v>Seven of Pentacles was checked open in the Russian tarot tracker before assignment. Art should show a rugged village laborer with stacked firewood, sled runners, repaired boundary posts, and exactly seven visible cut log ends, carved post marks, or pentacle-like wood rounds as the tarot cue.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="7" t="str">
-        <x:v>Six of Pentacles</x:v>
+        <x:v>Eight of Pentacles</x:v>
       </x:c>
       <x:c r="B79" s="7" t="str">
-        <x:v>Civilian Evacuee / Anya Petrovna</x:v>
+        <x:v>Yakov Antonov / Winter Engineer</x:v>
       </x:c>
       <x:c r="C79" s="7" t="str">
         <x:v>Winter Front</x:v>
@@ -2437,8 +2481,8 @@
         <x:v>Character</x:v>
       </x:c>
       <x:c r="E79" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/anya-petrovna-civilian-evacuee-six-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F79" s="7" t="str">
         <x:v>Saved</x:v>
@@ -2449,56 +2493,51 @@
       <x:c r="H79" s="7" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="I79" s="8" t="str">
-        <x:v>Card art shows Anya at a frozen evacuation road with a civilian sled, shared bread, a cracked icon with subtle reactor-red reflection, exactly six visible ration tokens, and a half-buried iron ring hinting at the later Deep North Circus connection. Six of Pentacles was checked open before assignment.</x:v>
-      </x:c>
+      <x:c r="I79" s="8" t="str"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="7" t="str">
-        <x:v>Seven of Pentacles</x:v>
+        <x:v>Nine of Pentacles</x:v>
       </x:c>
       <x:c r="B80" s="7" t="str">
-        <x:v>Village Woodcutter / Tomas Yurin</x:v>
+        <x:v>Cosmonaut Helmet With A Second Shadow</x:v>
       </x:c>
       <x:c r="C80" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D80" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E80" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/tomas-yurin-village-woodcutter-seven-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F80" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G80" s="7" t="str">
-        <x:v>Mapped</x:v>
+        <x:v>Unique</x:v>
       </x:c>
       <x:c r="H80" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I80" s="8" t="str">
-        <x:v>Seven of Pentacles was checked open in the Russian tarot tracker before assignment. Art should show a rugged village laborer with stacked firewood, sled runners, repaired boundary posts, and exactly seven visible cut log ends, carved post marks, or pentacle-like wood rounds as the tarot cue.</x:v>
+        <x:v>Approved</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="7" t="str">
-        <x:v>Eight of Pentacles</x:v>
+        <x:v>Ten of Pentacles</x:v>
       </x:c>
       <x:c r="B81" s="7" t="str">
-        <x:v>Yakov Antonov / Winter Engineer</x:v>
+        <x:v>The First Card Appears</x:v>
       </x:c>
       <x:c r="C81" s="7" t="str">
-        <x:v>Winter Front</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D81" s="7" t="str">
-        <x:v>Character</x:v>
+        <x:v>Event</x:v>
       </x:c>
       <x:c r="E81" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/yakov-antonov-winter-engineer-eight-of-pentacles-character-card-art-v2.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-ten-of-pentacles-event-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-ten-of-pentacles-event-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F81" s="7" t="str">
         <x:v>Saved</x:v>
@@ -2507,53 +2546,56 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H81" s="7" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="I81" s="8" t="str"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="7" t="str">
-        <x:v>Nine of Pentacles</x:v>
+        <x:v>Page of Pentacles</x:v>
       </x:c>
       <x:c r="B82" s="7" t="str">
-        <x:v>Cosmonaut Helmet With A Second Shadow</x:v>
+        <x:v>Sky-Hide Mirror</x:v>
       </x:c>
       <x:c r="C82" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D82" s="7" t="str">
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E82" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-pentacles-relic-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-cosmonaut-helmet-second-shadow-nine-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F82" s="7" t="str">
         <x:v>Saved</x:v>
       </x:c>
       <x:c r="G82" s="7" t="str">
-        <x:v>Unique</x:v>
+        <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H82" s="7" t="str">
-        <x:v>Approved</x:v>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I82" s="8" t="str">
+        <x:v>Remapped from Page of Cups to Page of Pentacles so Meteor Contact To The North can own the cup-message archetype. Corrected variant increases the mirror scale to match Pavel's character artwork, making it a large hand-held disc rather than a small pendant.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="7" t="str">
-        <x:v>Ten of Pentacles</x:v>
+        <x:v>Knight of Pentacles</x:v>
       </x:c>
       <x:c r="B83" s="7" t="str">
-        <x:v>The First Card Appears</x:v>
+        <x:v>Buran's Boundary Harness</x:v>
       </x:c>
       <x:c r="C83" s="7" t="str">
-        <x:v>Closed City</x:v>
+        <x:v>Far North</x:v>
       </x:c>
       <x:c r="D83" s="7" t="str">
-        <x:v>Event</x:v>
+        <x:v>Relic</x:v>
       </x:c>
       <x:c r="E83" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-ten-of-pentacles-event-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/events/closed-city-the-first-card-appears-ten-of-pentacles-event-art.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F83" s="7" t="str">
         <x:v>Saved</x:v>
@@ -2562,26 +2604,28 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H83" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I83" s="8" t="str"/>
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="I83" s="8" t="str">
+        <x:v>Relic art keeps the harness consistent with Buran and Vera's established imagery: rugged dark leather, iron rings, red cords, boundary charms, tiger pawprints, Vera's boot tracks, and aurora-lit village posts.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="7" t="str">
-        <x:v>Page of Pentacles</x:v>
+        <x:v>Queen of Pentacles</x:v>
       </x:c>
       <x:c r="B84" s="7" t="str">
-        <x:v>Sky-Hide Mirror</x:v>
+        <x:v>VERA-7</x:v>
       </x:c>
       <x:c r="C84" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D84" s="7" t="str">
-        <x:v>Relic</x:v>
+        <x:v>Character</x:v>
       </x:c>
       <x:c r="E84" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-sky-hide-mirror-page-of-cups-relic-art-corrected.png, friendlyName=Open art</x:v>
+        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-queen-of-pentacles-character-card-art.png","Open art")</x:f>
+        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-queen-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
       </x:c>
       <x:c r="F84" s="7" t="str">
         <x:v>Saved</x:v>
@@ -2590,97 +2634,37 @@
         <x:v>Mapped</x:v>
       </x:c>
       <x:c r="H84" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I84" s="8" t="str">
-        <x:v>Remapped from Page of Cups to Page of Pentacles so Meteor Contact To The North can own the cup-message archetype. Corrected variant increases the mirror scale to match Pavel's character artwork, making it a large hand-held disc rather than a small pendant.</x:v>
-      </x:c>
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="I84" s="8" t="str"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="7" t="str">
-        <x:v>Knight of Pentacles</x:v>
+        <x:v>King of Pentacles</x:v>
       </x:c>
       <x:c r="B85" s="7" t="str">
-        <x:v>Buran's Boundary Harness</x:v>
+        <x:v>Reactor Core Fragment</x:v>
       </x:c>
       <x:c r="C85" s="7" t="str">
-        <x:v>Far North</x:v>
+        <x:v>Closed City</x:v>
       </x:c>
       <x:c r="D85" s="7" t="str">
         <x:v>Relic</x:v>
       </x:c>
       <x:c r="E85" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/far-north-burans-boundary-harness-knight-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
-      </x:c>
-      <x:c r="F85" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G85" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H85" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="I85" s="8" t="str">
-        <x:v>Relic art keeps the harness consistent with Buran and Vera's established imagery: rugged dark leather, iron rings, red cords, boundary charms, tiger pawprints, Vera's boot tracks, and aurora-lit village posts.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="23" customHeight="1">
-      <x:c r="A86" s="7" t="str">
-        <x:v>Queen of Pentacles</x:v>
-      </x:c>
-      <x:c r="B86" s="7" t="str">
-        <x:v>VERA-7</x:v>
-      </x:c>
-      <x:c r="C86" s="7" t="str">
-        <x:v>Closed City</x:v>
-      </x:c>
-      <x:c r="D86" s="7" t="str">
-        <x:v>Character</x:v>
-      </x:c>
-      <x:c r="E86" s="9" t="e">
-        <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-queen-of-pentacles-character-card-art.png","Open art")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/characters/vera-7-queen-of-pentacles-character-card-art.png, friendlyName=Open art</x:v>
-      </x:c>
-      <x:c r="F86" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G86" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H86" s="7" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I86" s="8" t="str"/>
-    </x:row>
-    <x:row r="87" ht="23" customHeight="1">
-      <x:c r="A87" s="7" t="str">
-        <x:v>King of Pentacles</x:v>
-      </x:c>
-      <x:c r="B87" s="7" t="str">
-        <x:v>Reactor Core Fragment</x:v>
-      </x:c>
-      <x:c r="C87" s="7" t="str">
-        <x:v>Closed City</x:v>
-      </x:c>
-      <x:c r="D87" s="7" t="str">
-        <x:v>Relic</x:v>
-      </x:c>
-      <x:c r="E87" s="9" t="e">
         <x:f>HYPERLINK("file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-reactor-core-fragment-king-of-pentacles-relic-art.png","Open art")</x:f>
         <x:v>HYPERLINK is not implemented. linkLocation=file:///C:/Users/Drew/Documents/MythCards/assets/relics/closed-city-reactor-core-fragment-king-of-pentacles-relic-art.png, friendlyName=Open art</x:v>
       </x:c>
-      <x:c r="F87" s="7" t="str">
-        <x:v>Saved</x:v>
-      </x:c>
-      <x:c r="G87" s="7" t="str">
-        <x:v>Mapped</x:v>
-      </x:c>
-      <x:c r="H87" s="7" t="str">
+      <x:c r="F85" s="7" t="str">
+        <x:v>Saved</x:v>
+      </x:c>
+      <x:c r="G85" s="7" t="str">
+        <x:v>Mapped</x:v>
+      </x:c>
+      <x:c r="H85" s="7" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="I87" s="8" t="str">
+      <x:c r="I85" s="8" t="str">
         <x:v>Approved revision preserves the shard but replaces the paired gauges with a locked power pedestal, a single pentacle seal, and conduits carrying its energy into the Closed City.</x:v>
       </x:c>
     </x:row>
@@ -2694,7 +2678,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbed1ef9dbbd34973"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea99f41f14f242ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>